<commit_message>
change to example and tested ingest to sqlite
</commit_message>
<xml_diff>
--- a/scripts/example_input/AW172_voorbeeld_GD.xlsx
+++ b/scripts/example_input/AW172_voorbeeld_GD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dupuits\Documents\_HKV\faalpaden\scripts\example_input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKA\sources\github\faalkansbeheer\scripts\example_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F6CBA4-6312-44C2-B363-07CE101709E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5FA78A-5437-44D1-99ED-ABE7DDF0954D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{AD979432-8D0D-462C-972B-AB828F23136F}"/>
+    <workbookView xWindow="33525" yWindow="2400" windowWidth="21600" windowHeight="11295" xr2:uid="{AD979432-8D0D-462C-972B-AB828F23136F}"/>
   </bookViews>
   <sheets>
     <sheet name="scenario1" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="51">
   <si>
     <t>Template:</t>
   </si>
@@ -207,6 +207,12 @@
   </si>
   <si>
     <t>graverij</t>
+  </si>
+  <si>
+    <t>dummy</t>
+  </si>
+  <si>
+    <t>DP150</t>
   </si>
 </sst>
 </file>
@@ -451,7 +457,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
@@ -473,6 +478,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="2" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="2" fillId="2" borderId="9" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -481,9 +487,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
-    <cellStyle name="Input" xfId="2" builtinId="20"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Invoer" xfId="2" builtinId="20"/>
+    <cellStyle name="Kop 1" xfId="1" builtinId="16"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
     <dxf>
@@ -893,18 +899,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B226C6F-F461-456A-80C1-D38C6F61A2F7}">
   <dimension ref="A1:M60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" customWidth="1"/>
-    <col min="3" max="3" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="16.453125" customWidth="1"/>
-    <col min="12" max="12" width="18.26953125" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="16.42578125" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -912,14 +918,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>30</v>
       </c>
       <c r="B4" s="19"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -960,38 +966,48 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="6" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="5">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5">
+        <v>300</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="6">
-        <v>100</v>
-      </c>
-      <c r="G6" s="6" t="s">
+      <c r="F6" s="5">
+        <v>300</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="6">
         <v>0.1</v>
       </c>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="8" t="s">
+      <c r="K6" s="6">
+        <v>150</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>47</v>
       </c>
@@ -999,32 +1015,32 @@
       <c r="C11" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="9">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9">
+      <c r="D11" s="8">
+        <v>1</v>
+      </c>
+      <c r="E11" s="8">
         <v>2</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="8">
         <v>3</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="8">
         <v>4</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="8">
         <v>5</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="8">
         <v>6</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="8">
         <v>7</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1034,33 +1050,33 @@
       <c r="C12" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="K12" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="9">
+    <row r="13" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
         <v>1</v>
       </c>
       <c r="B13" t="s">
@@ -1069,21 +1085,21 @@
       <c r="C13" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-    </row>
-    <row r="14" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="9">
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
         <v>2</v>
       </c>
       <c r="B14" t="s">
@@ -1092,21 +1108,21 @@
       <c r="C14" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-    </row>
-    <row r="15" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="9">
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+    </row>
+    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
         <v>3</v>
       </c>
       <c r="B15" t="s">
@@ -1115,21 +1131,21 @@
       <c r="C15" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-    </row>
-    <row r="16" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="9">
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
         <v>4</v>
       </c>
       <c r="B16" t="s">
@@ -1138,72 +1154,72 @@
       <c r="C16" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="9">
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
         <v>5</v>
       </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A18" s="9">
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="8">
         <v>6</v>
       </c>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A19" s="9">
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="8">
         <v>7</v>
       </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A20" s="9">
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="8">
         <v>8</v>
       </c>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>31</v>
       </c>
@@ -1215,7 +1231,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -1241,7 +1257,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1</v>
       </c>
@@ -1262,12 +1278,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>9.9644263169334635E-8</v>
       </c>
-      <c r="H26" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H26" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1</v>
       </c>
@@ -1288,12 +1304,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>3.3976731247300535E-6</v>
       </c>
-      <c r="H27" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H27" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1</v>
       </c>
@@ -1314,12 +1330,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>1.5910859015753364E-4</v>
       </c>
-      <c r="H28" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H28" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1</v>
       </c>
@@ -1340,12 +1356,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>3.369292656768808E-4</v>
       </c>
-      <c r="H29" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H29" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1</v>
       </c>
@@ -1366,12 +1382,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2209605742717375E-16</v>
       </c>
-      <c r="H30" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H30" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1</v>
       </c>
@@ -1392,12 +1408,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>3.1671241833119857E-5</v>
       </c>
-      <c r="H31" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H31" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1</v>
       </c>
@@ -1418,12 +1434,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>0.5</v>
       </c>
-      <c r="H32" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H32" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1</v>
       </c>
@@ -1437,19 +1453,19 @@
       <c r="D33">
         <v>5.4</v>
       </c>
-      <c r="F33">
-        <v>8</v>
-      </c>
-      <c r="G33">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v>6.2209605742717375E-16</v>
-      </c>
-      <c r="H33" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="G33" t="str">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v/>
+      </c>
+      <c r="H33" s="16" t="e">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>3</v>
       </c>
@@ -1470,12 +1486,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>4.7918327659031834E-7</v>
       </c>
-      <c r="H34" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H34" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>3</v>
       </c>
@@ -1496,12 +1512,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2096653257761331E-3</v>
       </c>
-      <c r="H35" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H35" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>3</v>
       </c>
@@ -1522,12 +1538,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2209605742717375E-16</v>
       </c>
-      <c r="H36" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H36" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>3</v>
       </c>
@@ -1548,12 +1564,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2209605742717375E-16</v>
       </c>
-      <c r="H37" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H37" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>3</v>
       </c>
@@ -1567,19 +1583,19 @@
       <c r="D38">
         <v>5.4</v>
       </c>
-      <c r="F38">
-        <v>-8</v>
-      </c>
-      <c r="G38">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v>0.99999999999999933</v>
-      </c>
-      <c r="H38" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="G38" t="str">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v/>
+      </c>
+      <c r="H38" s="16" t="e">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2</v>
       </c>
@@ -1600,12 +1616,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2096653257761331E-3</v>
       </c>
-      <c r="H39" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H39" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2</v>
       </c>
@@ -1626,12 +1642,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2096653257761331E-3</v>
       </c>
-      <c r="H40" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H40" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2</v>
       </c>
@@ -1652,12 +1668,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>6.2209605742717375E-16</v>
       </c>
-      <c r="H41" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H41" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2</v>
       </c>
@@ -1678,12 +1694,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v>3.1671241833119857E-5</v>
       </c>
-      <c r="H42" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H42" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>4</v>
       </c>
@@ -1697,19 +1713,19 @@
       <c r="D43">
         <v>2</v>
       </c>
-      <c r="F43">
-        <v>-8</v>
-      </c>
-      <c r="G43">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v>0.99999999999999933</v>
-      </c>
-      <c r="H43" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="G43" t="str">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v/>
+      </c>
+      <c r="H43" s="16" t="e">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>4</v>
       </c>
@@ -1723,19 +1739,19 @@
       <c r="D44">
         <v>5.4</v>
       </c>
-      <c r="F44">
-        <v>-8</v>
-      </c>
-      <c r="G44">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v>0.99999999999999933</v>
-      </c>
-      <c r="H44" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="G44" t="str">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v/>
+      </c>
+      <c r="H44" s="16" t="e">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>4</v>
       </c>
@@ -1749,19 +1765,19 @@
       <c r="D45">
         <v>3</v>
       </c>
-      <c r="F45">
-        <v>-8</v>
-      </c>
-      <c r="G45">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v>0.99999999999999933</v>
-      </c>
-      <c r="H45" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="G45" t="str">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v/>
+      </c>
+      <c r="H45" s="16" t="e">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C46" t="str" cm="1">
         <f t="array" ref="C46">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1770,12 +1786,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H46" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H46" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C47" t="str" cm="1">
         <f t="array" ref="C47">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1784,12 +1800,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H47" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H47" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C48" t="str" cm="1">
         <f t="array" ref="C48">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1798,12 +1814,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H48" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H48" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C49" t="str" cm="1">
         <f t="array" ref="C49">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1812,12 +1828,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H49" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H49" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C50" t="str" cm="1">
         <f t="array" ref="C50">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1826,12 +1842,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H50" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H50" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C51" t="str" cm="1">
         <f t="array" ref="C51">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1840,12 +1856,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H51" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H51" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C52" t="str" cm="1">
         <f t="array" ref="C52">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1854,12 +1870,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H52" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H52" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C53" t="str" cm="1">
         <f t="array" ref="C53">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1868,12 +1884,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H53" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H53" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C54" t="str" cm="1">
         <f t="array" ref="C54">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1882,12 +1898,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H54" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H54" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C55" t="str" cm="1">
         <f t="array" ref="C55">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1896,12 +1912,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H55" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H55" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C56" t="str" cm="1">
         <f t="array" ref="C56">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1910,12 +1926,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H56" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H56" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C57" t="str" cm="1">
         <f t="array" ref="C57">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1924,12 +1940,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H57" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H57" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C58" t="str" cm="1">
         <f t="array" ref="C58">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1938,12 +1954,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H58" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H58" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C59" t="str" cm="1">
         <f t="array" ref="C59">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1952,12 +1968,12 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H59" s="17" t="str">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="H59" s="16" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C60" t="str" cm="1">
         <f t="array" ref="C60">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1966,7 +1982,7 @@
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H60" s="17" t="str">
+      <c r="H60" s="16" t="str">
         <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
         <v/>
       </c>
@@ -1989,43 +2005,43 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61B64AFC-FBDB-4219-8395-2E0D7C3338C5}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="13">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="12">
         <v>0</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="13"/>
-      <c r="B3" s="14"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="12"/>
+      <c r="B5" s="13"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="13"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="14"/>
+      <c r="B7" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2035,47 +2051,47 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2419547D-6BF3-46B8-ABC6-464DCDFC1905}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="13">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="12">
         <v>2.5</v>
       </c>
-      <c r="B2" s="18">
+      <c r="B2" s="17">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="13">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="12">
         <v>5.4</v>
       </c>
-      <c r="B3" s="18">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
+      <c r="B3" s="17">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="12"/>
+      <c r="B5" s="13"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="13"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="14"/>
+      <c r="B7" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>